<commit_message>
Add points for 8muyl6d5ahy04fbwarplcg3kk_playerlog
</commit_message>
<xml_diff>
--- a/bnc-streamlit-app/data/points/8muyl6d5ahy04fbwarplcg3kk_playerlog.xlsx
+++ b/bnc-streamlit-app/data/points/8muyl6d5ahy04fbwarplcg3kk_playerlog.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BG31"/>
+  <dimension ref="A1:BG33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -780,14 +780,14 @@
         </is>
       </c>
       <c r="N2" t="n">
-        <v>65</v>
+        <v>98</v>
       </c>
       <c r="O2" t="inlineStr"/>
       <c r="P2" t="n">
         <v>0</v>
       </c>
       <c r="Q2" t="n">
-        <v>65</v>
+        <v>98</v>
       </c>
       <c r="R2" t="inlineStr">
         <is>
@@ -795,7 +795,7 @@
         </is>
       </c>
       <c r="S2" t="n">
-        <v>65</v>
+        <v>98</v>
       </c>
       <c r="T2" t="inlineStr"/>
       <c r="U2" t="inlineStr"/>
@@ -835,7 +835,7 @@
         <v>0</v>
       </c>
       <c r="AM2" t="n">
-        <v>65</v>
+        <v>98</v>
       </c>
       <c r="AN2" t="n">
         <v>0</v>
@@ -951,7 +951,7 @@
         </is>
       </c>
       <c r="N3" t="n">
-        <v>65</v>
+        <v>98</v>
       </c>
       <c r="O3" t="inlineStr">
         <is>
@@ -962,7 +962,7 @@
         <v>0</v>
       </c>
       <c r="Q3" t="n">
-        <v>65</v>
+        <v>98</v>
       </c>
       <c r="R3" t="inlineStr">
         <is>
@@ -978,7 +978,7 @@
         </is>
       </c>
       <c r="U3" t="n">
-        <v>5</v>
+        <v>38</v>
       </c>
       <c r="V3" t="inlineStr"/>
       <c r="W3" t="inlineStr"/>
@@ -1014,21 +1014,21 @@
         </is>
       </c>
       <c r="AI3" t="n">
-        <v>-0.6182228200000001</v>
+        <v>-0.48988487</v>
       </c>
       <c r="AJ3" t="inlineStr">
         <is>
-          <t>-1.06</t>
+          <t>-1.00</t>
         </is>
       </c>
       <c r="AK3" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="AL3" t="n">
         <v>0</v>
       </c>
       <c r="AM3" t="n">
-        <v>65</v>
+        <v>98</v>
       </c>
       <c r="AN3" t="n">
         <v>0</v>
@@ -1052,7 +1052,7 @@
         <v>1</v>
       </c>
       <c r="AU3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AV3" t="n">
         <v>1</v>
@@ -1144,7 +1144,7 @@
         </is>
       </c>
       <c r="N4" t="n">
-        <v>65</v>
+        <v>98</v>
       </c>
       <c r="O4" t="inlineStr">
         <is>
@@ -1155,7 +1155,7 @@
         <v>0</v>
       </c>
       <c r="Q4" t="n">
-        <v>65</v>
+        <v>98</v>
       </c>
       <c r="R4" t="inlineStr">
         <is>
@@ -1171,7 +1171,7 @@
         </is>
       </c>
       <c r="U4" t="n">
-        <v>5</v>
+        <v>38</v>
       </c>
       <c r="V4" t="inlineStr"/>
       <c r="W4" t="inlineStr"/>
@@ -1207,21 +1207,21 @@
         </is>
       </c>
       <c r="AI4" t="n">
-        <v>-0.6186729800000002</v>
+        <v>-0.61838704</v>
       </c>
       <c r="AJ4" t="inlineStr">
         <is>
-          <t>-1.06</t>
+          <t>-1.13</t>
         </is>
       </c>
       <c r="AK4" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="AL4" t="n">
         <v>0</v>
       </c>
       <c r="AM4" t="n">
-        <v>65</v>
+        <v>98</v>
       </c>
       <c r="AN4" t="n">
         <v>0</v>
@@ -1233,7 +1233,7 @@
         <v>0</v>
       </c>
       <c r="AQ4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AR4" t="n">
         <v>4</v>
@@ -1242,7 +1242,7 @@
         <v>2</v>
       </c>
       <c r="AT4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AU4" t="n">
         <v>0</v>
@@ -1276,7 +1276,7 @@
         <v>0</v>
       </c>
       <c r="BF4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="BG4" t="n">
         <v>0</v>
@@ -1337,7 +1337,7 @@
         </is>
       </c>
       <c r="N5" t="n">
-        <v>65</v>
+        <v>98</v>
       </c>
       <c r="O5" t="inlineStr">
         <is>
@@ -1348,7 +1348,7 @@
         <v>0</v>
       </c>
       <c r="Q5" t="n">
-        <v>65</v>
+        <v>98</v>
       </c>
       <c r="R5" t="inlineStr">
         <is>
@@ -1364,7 +1364,7 @@
         </is>
       </c>
       <c r="U5" t="n">
-        <v>5</v>
+        <v>38</v>
       </c>
       <c r="V5" t="inlineStr"/>
       <c r="W5" t="inlineStr"/>
@@ -1400,21 +1400,21 @@
         </is>
       </c>
       <c r="AI5" t="n">
-        <v>-0.59614247</v>
+        <v>-0.60271827</v>
       </c>
       <c r="AJ5" t="inlineStr">
         <is>
-          <t>-1.04</t>
+          <t>-1.11</t>
         </is>
       </c>
       <c r="AK5" t="n">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="AL5" t="n">
         <v>0</v>
       </c>
       <c r="AM5" t="n">
-        <v>65</v>
+        <v>98</v>
       </c>
       <c r="AN5" t="n">
         <v>0</v>
@@ -1429,13 +1429,13 @@
         <v>0</v>
       </c>
       <c r="AR5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AS5" t="n">
         <v>4</v>
       </c>
       <c r="AT5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU5" t="n">
         <v>2</v>
@@ -1530,7 +1530,7 @@
         </is>
       </c>
       <c r="N6" t="n">
-        <v>65</v>
+        <v>98</v>
       </c>
       <c r="O6" t="inlineStr">
         <is>
@@ -1541,7 +1541,7 @@
         <v>0</v>
       </c>
       <c r="Q6" t="n">
-        <v>65</v>
+        <v>98</v>
       </c>
       <c r="R6" t="inlineStr">
         <is>
@@ -1557,7 +1557,7 @@
         </is>
       </c>
       <c r="U6" t="n">
-        <v>5</v>
+        <v>38</v>
       </c>
       <c r="V6" t="inlineStr"/>
       <c r="W6" t="inlineStr"/>
@@ -1593,40 +1593,40 @@
         </is>
       </c>
       <c r="AI6" t="n">
-        <v>0.2968530699999999</v>
+        <v>0.8199225499999999</v>
       </c>
       <c r="AJ6" t="inlineStr">
         <is>
-          <t>-0.15</t>
+          <t>+0.31</t>
         </is>
       </c>
       <c r="AK6" t="n">
+        <v>10</v>
+      </c>
+      <c r="AL6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM6" t="n">
+        <v>98</v>
+      </c>
+      <c r="AN6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ6" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR6" t="n">
+        <v>1</v>
+      </c>
+      <c r="AS6" t="n">
         <v>12</v>
       </c>
-      <c r="AL6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AM6" t="n">
-        <v>65</v>
-      </c>
-      <c r="AN6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AO6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AP6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AQ6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AR6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AS6" t="n">
-        <v>7</v>
-      </c>
       <c r="AT6" t="n">
         <v>2</v>
       </c>
@@ -1634,7 +1634,7 @@
         <v>1</v>
       </c>
       <c r="AV6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AW6" t="n">
         <v>0</v>
@@ -1782,11 +1782,11 @@
       </c>
       <c r="AJ7" t="inlineStr">
         <is>
-          <t>-0.70</t>
+          <t>-0.76</t>
         </is>
       </c>
       <c r="AK7" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="AL7" t="n">
         <v>0</v>
@@ -1967,11 +1967,11 @@
       </c>
       <c r="AJ8" t="inlineStr">
         <is>
-          <t>-0.60</t>
+          <t>-0.67</t>
         </is>
       </c>
       <c r="AK8" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="AL8" t="n">
         <v>0</v>
@@ -2152,11 +2152,11 @@
       </c>
       <c r="AJ9" t="inlineStr">
         <is>
-          <t>-0.50</t>
+          <t>-0.56</t>
         </is>
       </c>
       <c r="AK9" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="AL9" t="n">
         <v>0</v>
@@ -2347,11 +2347,11 @@
       </c>
       <c r="AJ10" t="inlineStr">
         <is>
-          <t>-0.30</t>
+          <t>-0.36</t>
         </is>
       </c>
       <c r="AK10" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="AL10" t="n">
         <v>0</v>
@@ -2459,10 +2459,12 @@
           <t>14dpnweb51v7re2xa3qkpulex</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr"/>
+      <c r="I11" t="n">
+        <v>2</v>
+      </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="K11" t="inlineStr"/>
@@ -2473,18 +2475,14 @@
         </is>
       </c>
       <c r="N11" t="n">
-        <v>65</v>
-      </c>
-      <c r="O11" t="inlineStr">
-        <is>
-          <t>RCM(2)</t>
-        </is>
-      </c>
+        <v>89</v>
+      </c>
+      <c r="O11" t="inlineStr"/>
       <c r="P11" t="n">
         <v>0</v>
       </c>
       <c r="Q11" t="n">
-        <v>65</v>
+        <v>89</v>
       </c>
       <c r="R11" t="inlineStr">
         <is>
@@ -2492,16 +2490,10 @@
         </is>
       </c>
       <c r="S11" t="n">
-        <v>60</v>
-      </c>
-      <c r="T11" t="inlineStr">
-        <is>
-          <t>RCM(2)</t>
-        </is>
-      </c>
-      <c r="U11" t="n">
-        <v>5</v>
-      </c>
+        <v>89</v>
+      </c>
+      <c r="T11" t="inlineStr"/>
+      <c r="U11" t="inlineStr"/>
       <c r="V11" t="inlineStr"/>
       <c r="W11" t="inlineStr"/>
       <c r="X11" t="inlineStr"/>
@@ -2528,7 +2520,7 @@
         <v>-0.2</v>
       </c>
       <c r="AG11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AH11" t="inlineStr">
         <is>
@@ -2536,21 +2528,21 @@
         </is>
       </c>
       <c r="AI11" t="n">
-        <v>0.03096378</v>
+        <v>0.20785925</v>
       </c>
       <c r="AJ11" t="inlineStr">
         <is>
-          <t>-0.41</t>
+          <t>-0.30</t>
         </is>
       </c>
       <c r="AK11" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="AL11" t="n">
         <v>0</v>
       </c>
       <c r="AM11" t="n">
-        <v>65</v>
+        <v>89</v>
       </c>
       <c r="AN11" t="n">
         <v>0</v>
@@ -2562,7 +2554,7 @@
         <v>0</v>
       </c>
       <c r="AQ11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AR11" t="n">
         <v>6</v>
@@ -2605,7 +2597,7 @@
         <v>0</v>
       </c>
       <c r="BF11" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="BG11" t="n">
         <v>0</v>
@@ -2666,14 +2658,18 @@
         </is>
       </c>
       <c r="N12" t="n">
-        <v>65</v>
-      </c>
-      <c r="O12" t="inlineStr"/>
+        <v>98</v>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>CF</t>
+        </is>
+      </c>
       <c r="P12" t="n">
         <v>0</v>
       </c>
       <c r="Q12" t="n">
-        <v>65</v>
+        <v>98</v>
       </c>
       <c r="R12" t="inlineStr">
         <is>
@@ -2681,10 +2677,16 @@
         </is>
       </c>
       <c r="S12" t="n">
-        <v>65</v>
-      </c>
-      <c r="T12" t="inlineStr"/>
-      <c r="U12" t="inlineStr"/>
+        <v>89.59999999999999</v>
+      </c>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>CF</t>
+        </is>
+      </c>
+      <c r="U12" t="n">
+        <v>8.4</v>
+      </c>
       <c r="V12" t="inlineStr"/>
       <c r="W12" t="inlineStr"/>
       <c r="X12" t="inlineStr"/>
@@ -2719,21 +2721,21 @@
         </is>
       </c>
       <c r="AI12" t="n">
-        <v>-0.40622991</v>
+        <v>-0.32220362</v>
       </c>
       <c r="AJ12" t="inlineStr">
         <is>
-          <t>-0.85</t>
+          <t>-0.83</t>
         </is>
       </c>
       <c r="AK12" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="AL12" t="n">
         <v>0</v>
       </c>
       <c r="AM12" t="n">
-        <v>65</v>
+        <v>98</v>
       </c>
       <c r="AN12" t="n">
         <v>0</v>
@@ -2745,7 +2747,7 @@
         <v>0</v>
       </c>
       <c r="AQ12" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AR12" t="n">
         <v>2</v>
@@ -2757,7 +2759,7 @@
         <v>0</v>
       </c>
       <c r="AU12" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AV12" t="n">
         <v>0</v>
@@ -2788,7 +2790,7 @@
         <v>0</v>
       </c>
       <c r="BF12" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="BG12" t="n">
         <v>0</v>
@@ -2807,17 +2809,17 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Alaa Al Hejji</t>
+          <t>Khalid Al Ghannam</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 18</t>
+          <t xml:space="preserve"> 17</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>RCB(3)</t>
+          <t>LCM(2)</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -2832,7 +2834,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>6wto8d6jcd41bo451wwbjng89</t>
+          <t>92qhzmz7bik9yiyhpt9fcvqzu</t>
         </is>
       </c>
       <c r="I13" t="inlineStr"/>
@@ -2842,7 +2844,7 @@
         </is>
       </c>
       <c r="K13" t="n">
-        <v>59</v>
+        <v>89</v>
       </c>
       <c r="L13" t="n">
         <v>2</v>
@@ -2853,34 +2855,34 @@
         </is>
       </c>
       <c r="N13" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="O13" t="inlineStr">
         <is>
+          <t>LM</t>
+        </is>
+      </c>
+      <c r="P13" t="n">
+        <v>89</v>
+      </c>
+      <c r="Q13" t="n">
+        <v>98</v>
+      </c>
+      <c r="R13" t="inlineStr">
+        <is>
           <t>LCM(2)</t>
         </is>
       </c>
-      <c r="P13" t="n">
-        <v>59</v>
-      </c>
-      <c r="Q13" t="n">
-        <v>65</v>
-      </c>
-      <c r="R13" t="inlineStr">
-        <is>
-          <t>RCB(3)</t>
-        </is>
-      </c>
       <c r="S13" t="n">
-        <v>1</v>
+        <v>0.6</v>
       </c>
       <c r="T13" t="inlineStr">
         <is>
-          <t>LCM(2)</t>
+          <t>LM</t>
         </is>
       </c>
       <c r="U13" t="n">
-        <v>5</v>
+        <v>8.4</v>
       </c>
       <c r="V13" t="inlineStr"/>
       <c r="W13" t="inlineStr"/>
@@ -2912,25 +2914,25 @@
       </c>
       <c r="AH13" t="inlineStr">
         <is>
-          <t>Alaa Al Hejji</t>
+          <t>Khalid Al Ghannam</t>
         </is>
       </c>
       <c r="AI13" t="n">
-        <v>-0.005348430000000001</v>
+        <v>0</v>
       </c>
       <c r="AJ13" t="inlineStr">
         <is>
-          <t>-0.45</t>
+          <t>-0.51</t>
         </is>
       </c>
       <c r="AK13" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="AL13" t="n">
-        <v>59</v>
+        <v>89</v>
       </c>
       <c r="AM13" t="n">
-        <v>65</v>
+        <v>98</v>
       </c>
       <c r="AN13" t="n">
         <v>0</v>
@@ -3004,17 +3006,17 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Abdullah Al Hamddan</t>
+          <t>Alaa Al Hejji</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 19</t>
+          <t xml:space="preserve"> 18</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>CF</t>
+          <t>RCB(3)</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -3029,7 +3031,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>hki3chjlidmwubff6srauj56</t>
+          <t>6wto8d6jcd41bo451wwbjng89</t>
         </is>
       </c>
       <c r="I14" t="inlineStr"/>
@@ -3039,7 +3041,7 @@
         </is>
       </c>
       <c r="K14" t="n">
-        <v>45</v>
+        <v>59</v>
       </c>
       <c r="L14" t="n">
         <v>2</v>
@@ -3050,25 +3052,35 @@
         </is>
       </c>
       <c r="N14" t="n">
-        <v>20</v>
-      </c>
-      <c r="O14" t="inlineStr"/>
+        <v>39</v>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>RCM(2)</t>
+        </is>
+      </c>
       <c r="P14" t="n">
-        <v>45</v>
+        <v>59</v>
       </c>
       <c r="Q14" t="n">
-        <v>65</v>
+        <v>98</v>
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>CF</t>
+          <t>RCB(3)</t>
         </is>
       </c>
       <c r="S14" t="n">
-        <v>20</v>
-      </c>
-      <c r="T14" t="inlineStr"/>
-      <c r="U14" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="T14" t="inlineStr">
+        <is>
+          <t>RCM(2)</t>
+        </is>
+      </c>
+      <c r="U14" t="n">
+        <v>38</v>
+      </c>
       <c r="V14" t="inlineStr"/>
       <c r="W14" t="inlineStr"/>
       <c r="X14" t="inlineStr"/>
@@ -3089,35 +3101,35 @@
         <v>0</v>
       </c>
       <c r="AE14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AF14" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AG14" t="n">
         <v>2</v>
       </c>
       <c r="AH14" t="inlineStr">
         <is>
-          <t>Abdullah Al Hamddan</t>
+          <t>Alaa Al Hejji</t>
         </is>
       </c>
       <c r="AI14" t="n">
-        <v>0.22627978</v>
+        <v>0.14432678</v>
       </c>
       <c r="AJ14" t="inlineStr">
         <is>
-          <t>-0.22</t>
+          <t>-0.36</t>
         </is>
       </c>
       <c r="AK14" t="n">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="AL14" t="n">
-        <v>90</v>
+        <v>59</v>
       </c>
       <c r="AM14" t="n">
-        <v>65</v>
+        <v>98</v>
       </c>
       <c r="AN14" t="n">
         <v>0</v>
@@ -3135,10 +3147,10 @@
         <v>0</v>
       </c>
       <c r="AS14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AT14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU14" t="n">
         <v>0</v>
@@ -3191,17 +3203,17 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Mohamed Kanno</t>
+          <t>Abdullah Al Hamddan</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 23</t>
+          <t xml:space="preserve"> 19</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>RCM(2)</t>
+          <t>CF</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
@@ -3216,7 +3228,7 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>d25hyz1ov3mdflbnbyc9okrmd</t>
+          <t>hki3chjlidmwubff6srauj56</t>
         </is>
       </c>
       <c r="I15" t="inlineStr"/>
@@ -3237,35 +3249,25 @@
         </is>
       </c>
       <c r="N15" t="n">
-        <v>20</v>
-      </c>
-      <c r="O15" t="inlineStr">
-        <is>
-          <t>CF</t>
-        </is>
-      </c>
+        <v>53</v>
+      </c>
+      <c r="O15" t="inlineStr"/>
       <c r="P15" t="n">
         <v>45</v>
       </c>
       <c r="Q15" t="n">
-        <v>65</v>
+        <v>98</v>
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>RCM(2)</t>
+          <t>CF</t>
         </is>
       </c>
       <c r="S15" t="n">
-        <v>15</v>
-      </c>
-      <c r="T15" t="inlineStr">
-        <is>
-          <t>CF</t>
-        </is>
-      </c>
-      <c r="U15" t="n">
-        <v>5</v>
-      </c>
+        <v>53</v>
+      </c>
+      <c r="T15" t="inlineStr"/>
+      <c r="U15" t="inlineStr"/>
       <c r="V15" t="inlineStr"/>
       <c r="W15" t="inlineStr"/>
       <c r="X15" t="inlineStr"/>
@@ -3289,32 +3291,32 @@
         <v>1</v>
       </c>
       <c r="AF15" t="n">
-        <v>-0.05</v>
+        <v>0</v>
       </c>
       <c r="AG15" t="n">
         <v>2</v>
       </c>
       <c r="AH15" t="inlineStr">
         <is>
-          <t>Mohamed Kanno</t>
+          <t>Abdullah Al Hamddan</t>
         </is>
       </c>
       <c r="AI15" t="n">
-        <v>-0.24776608</v>
+        <v>0.57243928</v>
       </c>
       <c r="AJ15" t="inlineStr">
         <is>
-          <t>-0.69</t>
+          <t>+0.07</t>
         </is>
       </c>
       <c r="AK15" t="n">
-        <v>23</v>
+        <v>12</v>
       </c>
       <c r="AL15" t="n">
         <v>90</v>
       </c>
       <c r="AM15" t="n">
-        <v>65</v>
+        <v>98</v>
       </c>
       <c r="AN15" t="n">
         <v>0</v>
@@ -3326,13 +3328,13 @@
         <v>0</v>
       </c>
       <c r="AQ15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AR15" t="n">
         <v>0</v>
       </c>
       <c r="AS15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AT15" t="n">
         <v>0</v>
@@ -3344,10 +3346,10 @@
         <v>0</v>
       </c>
       <c r="AW15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AX15" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AY15" t="n">
         <v>0</v>
@@ -3369,7 +3371,7 @@
         <v>0</v>
       </c>
       <c r="BF15" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="BG15" t="n">
         <v>0</v>
@@ -3388,17 +3390,17 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Mohammed Abu Al Shamat</t>
+          <t>Mohamed Kanno</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 26</t>
+          <t xml:space="preserve"> 23</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>CF</t>
+          <t>RCM(2)</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -3413,7 +3415,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>3oweqcxu9yiunzz29vpi5kro4</t>
+          <t>d25hyz1ov3mdflbnbyc9okrmd</t>
         </is>
       </c>
       <c r="I16" t="inlineStr"/>
@@ -3423,7 +3425,7 @@
         </is>
       </c>
       <c r="K16" t="n">
-        <v>59</v>
+        <v>45</v>
       </c>
       <c r="L16" t="n">
         <v>2</v>
@@ -3434,37 +3436,43 @@
         </is>
       </c>
       <c r="N16" t="n">
-        <v>6</v>
+        <v>53</v>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>RM</t>
+          <t>CF, LCM(2)</t>
         </is>
       </c>
       <c r="P16" t="n">
-        <v>59</v>
+        <v>45</v>
       </c>
       <c r="Q16" t="n">
-        <v>65</v>
+        <v>98</v>
       </c>
       <c r="R16" t="inlineStr">
         <is>
+          <t>RCM(2)</t>
+        </is>
+      </c>
+      <c r="S16" t="n">
+        <v>15</v>
+      </c>
+      <c r="T16" t="inlineStr">
+        <is>
           <t>CF</t>
         </is>
       </c>
-      <c r="S16" t="n">
-        <v>1</v>
-      </c>
-      <c r="T16" t="inlineStr">
-        <is>
-          <t>RM</t>
-        </is>
-      </c>
       <c r="U16" t="n">
-        <v>5</v>
-      </c>
-      <c r="V16" t="inlineStr"/>
-      <c r="W16" t="inlineStr"/>
+        <v>29.6</v>
+      </c>
+      <c r="V16" t="inlineStr">
+        <is>
+          <t>LCM(2)</t>
+        </is>
+      </c>
+      <c r="W16" t="n">
+        <v>8.4</v>
+      </c>
       <c r="X16" t="inlineStr"/>
       <c r="Y16" t="inlineStr"/>
       <c r="Z16" t="inlineStr"/>
@@ -3483,35 +3491,35 @@
         <v>0</v>
       </c>
       <c r="AE16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AF16" t="n">
-        <v>0</v>
+        <v>-0.05</v>
       </c>
       <c r="AG16" t="n">
         <v>2</v>
       </c>
       <c r="AH16" t="inlineStr">
         <is>
-          <t>Mohammed Abu Al Shamat</t>
+          <t>Mohamed Kanno</t>
         </is>
       </c>
       <c r="AI16" t="n">
-        <v>0.0001119200000000015</v>
+        <v>-0.1375335600000001</v>
       </c>
       <c r="AJ16" t="inlineStr">
         <is>
-          <t>-0.44</t>
+          <t>-0.64</t>
         </is>
       </c>
       <c r="AK16" t="n">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="AL16" t="n">
-        <v>59</v>
+        <v>90</v>
       </c>
       <c r="AM16" t="n">
-        <v>65</v>
+        <v>98</v>
       </c>
       <c r="AN16" t="n">
         <v>0</v>
@@ -3526,7 +3534,7 @@
         <v>0</v>
       </c>
       <c r="AR16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AS16" t="n">
         <v>0</v>
@@ -3544,7 +3552,7 @@
         <v>0</v>
       </c>
       <c r="AX16" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AY16" t="n">
         <v>0</v>
@@ -3580,37 +3588,37 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>eh7yt2x2wck51oixw8012ux5j</t>
+          <t>9l4imoomrnyceg5u3kdxf5l5r</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Unai Simón</t>
+          <t>Mohammed Abu Al Shamat</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>23</t>
+          <t xml:space="preserve"> 26</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>GK</t>
+          <t>CF</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>4vlurpsi44g09g159t61u83bp</t>
+          <t>3oweqcxu9yiunzz29vpi5kro4</t>
         </is>
       </c>
       <c r="I17" t="inlineStr"/>
@@ -3619,33 +3627,47 @@
           <t>no</t>
         </is>
       </c>
-      <c r="K17" t="inlineStr"/>
-      <c r="L17" t="inlineStr"/>
+      <c r="K17" t="n">
+        <v>59</v>
+      </c>
+      <c r="L17" t="n">
+        <v>2</v>
+      </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="N17" t="n">
-        <v>65</v>
-      </c>
-      <c r="O17" t="inlineStr"/>
+        <v>39</v>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>RM</t>
+        </is>
+      </c>
       <c r="P17" t="n">
-        <v>0</v>
+        <v>59</v>
       </c>
       <c r="Q17" t="n">
-        <v>65</v>
+        <v>98</v>
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>GK</t>
+          <t>CF</t>
         </is>
       </c>
       <c r="S17" t="n">
-        <v>65</v>
-      </c>
-      <c r="T17" t="inlineStr"/>
-      <c r="U17" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="T17" t="inlineStr">
+        <is>
+          <t>RM</t>
+        </is>
+      </c>
+      <c r="U17" t="n">
+        <v>38</v>
+      </c>
       <c r="V17" t="inlineStr"/>
       <c r="W17" t="inlineStr"/>
       <c r="X17" t="inlineStr"/>
@@ -3654,16 +3676,16 @@
       <c r="AA17" t="inlineStr"/>
       <c r="AB17" t="inlineStr">
         <is>
-          <t>eh7yt2x2wck51oixw8012ux5j</t>
+          <t>9l4imoomrnyceg5u3kdxf5l5r</t>
         </is>
       </c>
       <c r="AC17" t="inlineStr">
         <is>
-          <t>Spain</t>
+          <t>Saudi Arabia</t>
         </is>
       </c>
       <c r="AD17" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="AE17" t="n">
         <v>0</v>
@@ -3672,17 +3694,29 @@
         <v>0</v>
       </c>
       <c r="AG17" t="n">
-        <v>1</v>
-      </c>
-      <c r="AH17" t="inlineStr"/>
-      <c r="AI17" t="inlineStr"/>
-      <c r="AJ17" t="inlineStr"/>
-      <c r="AK17" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="AH17" t="inlineStr">
+        <is>
+          <t>Mohammed Abu Al Shamat</t>
+        </is>
+      </c>
+      <c r="AI17" t="n">
+        <v>0.18696528</v>
+      </c>
+      <c r="AJ17" t="inlineStr">
+        <is>
+          <t>-0.32</t>
+        </is>
+      </c>
+      <c r="AK17" t="n">
+        <v>16</v>
+      </c>
       <c r="AL17" t="n">
-        <v>0</v>
+        <v>59</v>
       </c>
       <c r="AM17" t="n">
-        <v>65</v>
+        <v>98</v>
       </c>
       <c r="AN17" t="n">
         <v>0</v>
@@ -3697,16 +3731,16 @@
         <v>0</v>
       </c>
       <c r="AR17" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="AS17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AT17" t="n">
         <v>0</v>
       </c>
       <c r="AU17" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AV17" t="n">
         <v>0</v>
@@ -3732,11 +3766,7 @@
       <c r="BC17" t="n">
         <v>0</v>
       </c>
-      <c r="BD17" t="inlineStr">
-        <is>
-          <t>GK</t>
-        </is>
-      </c>
+      <c r="BD17" t="inlineStr"/>
       <c r="BE17" t="n">
         <v>0</v>
       </c>
@@ -3744,7 +3774,7 @@
         <v>0</v>
       </c>
       <c r="BG17" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18">
@@ -3760,17 +3790,17 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Pedro Porro</t>
+          <t>Unai Simón</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 12</t>
+          <t>23</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>RB</t>
+          <t>GK</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -3780,12 +3810,12 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>77yaqzy45dxtzicao00jxrlgq</t>
+          <t>4vlurpsi44g09g159t61u83bp</t>
         </is>
       </c>
       <c r="I18" t="inlineStr"/>
@@ -3802,22 +3832,22 @@
         </is>
       </c>
       <c r="N18" t="n">
-        <v>65</v>
+        <v>98</v>
       </c>
       <c r="O18" t="inlineStr"/>
       <c r="P18" t="n">
         <v>0</v>
       </c>
       <c r="Q18" t="n">
-        <v>65</v>
+        <v>98</v>
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>RB</t>
+          <t>GK</t>
         </is>
       </c>
       <c r="S18" t="n">
-        <v>65</v>
+        <v>98</v>
       </c>
       <c r="T18" t="inlineStr"/>
       <c r="U18" t="inlineStr"/>
@@ -3844,32 +3874,20 @@
         <v>0</v>
       </c>
       <c r="AF18" t="n">
-        <v>0.4</v>
+        <v>0</v>
       </c>
       <c r="AG18" t="n">
         <v>1</v>
       </c>
-      <c r="AH18" t="inlineStr">
-        <is>
-          <t>Pedro Porro</t>
-        </is>
-      </c>
-      <c r="AI18" t="n">
-        <v>1.73661249</v>
-      </c>
-      <c r="AJ18" t="inlineStr">
-        <is>
-          <t>+1.29</t>
-        </is>
-      </c>
-      <c r="AK18" t="n">
-        <v>3</v>
-      </c>
+      <c r="AH18" t="inlineStr"/>
+      <c r="AI18" t="inlineStr"/>
+      <c r="AJ18" t="inlineStr"/>
+      <c r="AK18" t="inlineStr"/>
       <c r="AL18" t="n">
         <v>0</v>
       </c>
       <c r="AM18" t="n">
-        <v>65</v>
+        <v>98</v>
       </c>
       <c r="AN18" t="n">
         <v>0</v>
@@ -3878,7 +3896,7 @@
         <v>0</v>
       </c>
       <c r="AP18" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AQ18" t="n">
         <v>0</v>
@@ -3890,16 +3908,16 @@
         <v>1</v>
       </c>
       <c r="AT18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AU18" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AV18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AW18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AX18" t="n">
         <v>0</v>
@@ -3921,17 +3939,17 @@
       </c>
       <c r="BD18" t="inlineStr">
         <is>
-          <t>DEF</t>
+          <t>GK</t>
         </is>
       </c>
       <c r="BE18" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="BF18" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="BG18" t="n">
-        <v>6</v>
+        <v>6.5</v>
       </c>
     </row>
     <row r="19">
@@ -3947,17 +3965,17 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Marc Cucurella</t>
+          <t>Pedro Porro</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 24</t>
+          <t xml:space="preserve"> 12</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>LB</t>
+          <t>RB</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
@@ -3967,12 +3985,12 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>7c2wnewpcf1idj6ghj6gu0wyd</t>
+          <t>77yaqzy45dxtzicao00jxrlgq</t>
         </is>
       </c>
       <c r="I19" t="inlineStr"/>
@@ -3989,22 +4007,22 @@
         </is>
       </c>
       <c r="N19" t="n">
-        <v>65</v>
+        <v>98</v>
       </c>
       <c r="O19" t="inlineStr"/>
       <c r="P19" t="n">
         <v>0</v>
       </c>
       <c r="Q19" t="n">
-        <v>65</v>
+        <v>98</v>
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>LB</t>
+          <t>RB</t>
         </is>
       </c>
       <c r="S19" t="n">
-        <v>65</v>
+        <v>98</v>
       </c>
       <c r="T19" t="inlineStr"/>
       <c r="U19" t="inlineStr"/>
@@ -4038,25 +4056,25 @@
       </c>
       <c r="AH19" t="inlineStr">
         <is>
-          <t>Marc Cucurella</t>
+          <t>Pedro Porro</t>
         </is>
       </c>
       <c r="AI19" t="n">
-        <v>1.20395353</v>
+        <v>1.87972255</v>
       </c>
       <c r="AJ19" t="inlineStr">
         <is>
-          <t>+0.76</t>
+          <t>+1.37</t>
         </is>
       </c>
       <c r="AK19" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="AL19" t="n">
         <v>0</v>
       </c>
       <c r="AM19" t="n">
-        <v>65</v>
+        <v>98</v>
       </c>
       <c r="AN19" t="n">
         <v>0</v>
@@ -4065,22 +4083,22 @@
         <v>0</v>
       </c>
       <c r="AP19" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AQ19" t="n">
         <v>0</v>
       </c>
       <c r="AR19" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="AS19" t="n">
         <v>2</v>
       </c>
       <c r="AT19" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AU19" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AV19" t="n">
         <v>0</v>
@@ -4112,10 +4130,10 @@
         </is>
       </c>
       <c r="BE19" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="BF19" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="BG19" t="n">
         <v>6</v>
@@ -4134,17 +4152,17 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Rodri</t>
+          <t>Marc Cucurella</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 16</t>
+          <t xml:space="preserve"> 24</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>CM(3)</t>
+          <t>LB</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -4154,12 +4172,12 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>dqfk7czrayirrvonirtk2mk15</t>
+          <t>7c2wnewpcf1idj6ghj6gu0wyd</t>
         </is>
       </c>
       <c r="I20" t="inlineStr"/>
@@ -4176,22 +4194,22 @@
         </is>
       </c>
       <c r="N20" t="n">
-        <v>65</v>
+        <v>98</v>
       </c>
       <c r="O20" t="inlineStr"/>
       <c r="P20" t="n">
         <v>0</v>
       </c>
       <c r="Q20" t="n">
-        <v>65</v>
+        <v>98</v>
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>CM(3)</t>
+          <t>LB</t>
         </is>
       </c>
       <c r="S20" t="n">
-        <v>65</v>
+        <v>98</v>
       </c>
       <c r="T20" t="inlineStr"/>
       <c r="U20" t="inlineStr"/>
@@ -4218,22 +4236,22 @@
         <v>0</v>
       </c>
       <c r="AF20" t="n">
-        <v>0.1</v>
+        <v>0.4</v>
       </c>
       <c r="AG20" t="n">
         <v>1</v>
       </c>
       <c r="AH20" t="inlineStr">
         <is>
-          <t>Rodri</t>
+          <t>Marc Cucurella</t>
         </is>
       </c>
       <c r="AI20" t="n">
-        <v>1.19777616</v>
+        <v>1.35047266</v>
       </c>
       <c r="AJ20" t="inlineStr">
         <is>
-          <t>+0.75</t>
+          <t>+0.84</t>
         </is>
       </c>
       <c r="AK20" t="n">
@@ -4243,7 +4261,7 @@
         <v>0</v>
       </c>
       <c r="AM20" t="n">
-        <v>65</v>
+        <v>98</v>
       </c>
       <c r="AN20" t="n">
         <v>0</v>
@@ -4252,13 +4270,13 @@
         <v>0</v>
       </c>
       <c r="AP20" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AQ20" t="n">
         <v>1</v>
       </c>
       <c r="AR20" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="AS20" t="n">
         <v>2</v>
@@ -4267,13 +4285,13 @@
         <v>1</v>
       </c>
       <c r="AU20" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AV20" t="n">
         <v>0</v>
       </c>
       <c r="AW20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AX20" t="n">
         <v>0</v>
@@ -4295,17 +4313,17 @@
       </c>
       <c r="BD20" t="inlineStr">
         <is>
-          <t>MID</t>
+          <t>DEF</t>
         </is>
       </c>
       <c r="BE20" t="n">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="BF20" t="n">
         <v>2</v>
       </c>
       <c r="BG20" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="21">
@@ -4321,17 +4339,17 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Pau Cubarsí</t>
+          <t>Rodri</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 22</t>
+          <t xml:space="preserve"> 16</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>RCB(2)</t>
+          <t>CM(3)</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -4341,12 +4359,12 @@
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>bkwxem45cf48k14euwqe7rs44</t>
+          <t>dqfk7czrayirrvonirtk2mk15</t>
         </is>
       </c>
       <c r="I21" t="inlineStr"/>
@@ -4363,22 +4381,22 @@
         </is>
       </c>
       <c r="N21" t="n">
-        <v>65</v>
+        <v>98</v>
       </c>
       <c r="O21" t="inlineStr"/>
       <c r="P21" t="n">
         <v>0</v>
       </c>
       <c r="Q21" t="n">
-        <v>65</v>
+        <v>98</v>
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>RCB(2)</t>
+          <t>CM(3)</t>
         </is>
       </c>
       <c r="S21" t="n">
-        <v>65</v>
+        <v>98</v>
       </c>
       <c r="T21" t="inlineStr"/>
       <c r="U21" t="inlineStr"/>
@@ -4405,94 +4423,94 @@
         <v>0</v>
       </c>
       <c r="AF21" t="n">
-        <v>0.4</v>
+        <v>0.1</v>
       </c>
       <c r="AG21" t="n">
         <v>1</v>
       </c>
       <c r="AH21" t="inlineStr">
         <is>
-          <t>Pau Cubarsí</t>
+          <t>Rodri</t>
         </is>
       </c>
       <c r="AI21" t="n">
-        <v>1.37476125</v>
+        <v>1.37263949</v>
       </c>
       <c r="AJ21" t="inlineStr">
         <is>
-          <t>+0.93</t>
+          <t>+0.87</t>
         </is>
       </c>
       <c r="AK21" t="n">
+        <v>6</v>
+      </c>
+      <c r="AL21" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM21" t="n">
+        <v>98</v>
+      </c>
+      <c r="AN21" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO21" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP21" t="n">
+        <v>1</v>
+      </c>
+      <c r="AQ21" t="n">
+        <v>1</v>
+      </c>
+      <c r="AR21" t="n">
+        <v>8</v>
+      </c>
+      <c r="AS21" t="n">
+        <v>2</v>
+      </c>
+      <c r="AT21" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU21" t="n">
+        <v>2</v>
+      </c>
+      <c r="AV21" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW21" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX21" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY21" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ21" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA21" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB21" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC21" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD21" t="inlineStr">
+        <is>
+          <t>MID</t>
+        </is>
+      </c>
+      <c r="BE21" t="n">
+        <v>13</v>
+      </c>
+      <c r="BF21" t="n">
+        <v>2</v>
+      </c>
+      <c r="BG21" t="n">
         <v>5</v>
-      </c>
-      <c r="AL21" t="n">
-        <v>0</v>
-      </c>
-      <c r="AM21" t="n">
-        <v>65</v>
-      </c>
-      <c r="AN21" t="n">
-        <v>0</v>
-      </c>
-      <c r="AO21" t="n">
-        <v>0</v>
-      </c>
-      <c r="AP21" t="n">
-        <v>2</v>
-      </c>
-      <c r="AQ21" t="n">
-        <v>0</v>
-      </c>
-      <c r="AR21" t="n">
-        <v>3</v>
-      </c>
-      <c r="AS21" t="n">
-        <v>2</v>
-      </c>
-      <c r="AT21" t="n">
-        <v>2</v>
-      </c>
-      <c r="AU21" t="n">
-        <v>0</v>
-      </c>
-      <c r="AV21" t="n">
-        <v>0</v>
-      </c>
-      <c r="AW21" t="n">
-        <v>0</v>
-      </c>
-      <c r="AX21" t="n">
-        <v>0</v>
-      </c>
-      <c r="AY21" t="n">
-        <v>0</v>
-      </c>
-      <c r="AZ21" t="n">
-        <v>0</v>
-      </c>
-      <c r="BA21" t="n">
-        <v>0</v>
-      </c>
-      <c r="BB21" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC21" t="n">
-        <v>0</v>
-      </c>
-      <c r="BD21" t="inlineStr">
-        <is>
-          <t>DEF</t>
-        </is>
-      </c>
-      <c r="BE21" t="n">
-        <v>4</v>
-      </c>
-      <c r="BF21" t="n">
-        <v>2</v>
-      </c>
-      <c r="BG21" t="n">
-        <v>6</v>
       </c>
     </row>
     <row r="22">
@@ -4508,17 +4526,17 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Aymeric Laporte</t>
+          <t>Pau Cubarsí</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 14</t>
+          <t xml:space="preserve"> 22</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>LCB(2)</t>
+          <t>RCB(2)</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -4528,12 +4546,12 @@
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>7fmpgkx58o9pivo2bbnxxkt05</t>
+          <t>bkwxem45cf48k14euwqe7rs44</t>
         </is>
       </c>
       <c r="I22" t="inlineStr"/>
@@ -4550,22 +4568,22 @@
         </is>
       </c>
       <c r="N22" t="n">
-        <v>65</v>
+        <v>98</v>
       </c>
       <c r="O22" t="inlineStr"/>
       <c r="P22" t="n">
         <v>0</v>
       </c>
       <c r="Q22" t="n">
-        <v>65</v>
+        <v>98</v>
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>LCB(2)</t>
+          <t>RCB(2)</t>
         </is>
       </c>
       <c r="S22" t="n">
-        <v>65</v>
+        <v>98</v>
       </c>
       <c r="T22" t="inlineStr"/>
       <c r="U22" t="inlineStr"/>
@@ -4599,49 +4617,49 @@
       </c>
       <c r="AH22" t="inlineStr">
         <is>
-          <t>Aymeric Laporte</t>
+          <t>Pau Cubarsí</t>
         </is>
       </c>
       <c r="AI22" t="n">
-        <v>1.54477156</v>
+        <v>1.50223305</v>
       </c>
       <c r="AJ22" t="inlineStr">
         <is>
-          <t>+1.10</t>
+          <t>+1.00</t>
         </is>
       </c>
       <c r="AK22" t="n">
+        <v>5</v>
+      </c>
+      <c r="AL22" t="n">
+        <v>0</v>
+      </c>
+      <c r="AM22" t="n">
+        <v>98</v>
+      </c>
+      <c r="AN22" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO22" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP22" t="n">
+        <v>2</v>
+      </c>
+      <c r="AQ22" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR22" t="n">
         <v>4</v>
       </c>
-      <c r="AL22" t="n">
-        <v>0</v>
-      </c>
-      <c r="AM22" t="n">
-        <v>65</v>
-      </c>
-      <c r="AN22" t="n">
-        <v>0</v>
-      </c>
-      <c r="AO22" t="n">
-        <v>1</v>
-      </c>
-      <c r="AP22" t="n">
-        <v>2</v>
-      </c>
-      <c r="AQ22" t="n">
-        <v>0</v>
-      </c>
-      <c r="AR22" t="n">
-        <v>1</v>
-      </c>
       <c r="AS22" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AT22" t="n">
         <v>2</v>
       </c>
       <c r="AU22" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AV22" t="n">
         <v>0</v>
@@ -4679,7 +4697,7 @@
         <v>2</v>
       </c>
       <c r="BG22" t="n">
-        <v>10</v>
+        <v>6</v>
       </c>
     </row>
     <row r="23">
@@ -4695,17 +4713,17 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Dani Olmo</t>
+          <t>Aymeric Laporte</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 10</t>
+          <t xml:space="preserve"> 14</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>RCM(3)</t>
+          <t>LCB(2)</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
@@ -4715,20 +4733,18 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>4gq1u1mqg0qzekh1u5djleeax</t>
-        </is>
-      </c>
-      <c r="I23" t="n">
-        <v>2</v>
-      </c>
+          <t>7fmpgkx58o9pivo2bbnxxkt05</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr"/>
       <c r="J23" t="inlineStr">
         <is>
-          <t>yes</t>
+          <t>no</t>
         </is>
       </c>
       <c r="K23" t="inlineStr"/>
@@ -4739,22 +4755,22 @@
         </is>
       </c>
       <c r="N23" t="n">
-        <v>60</v>
+        <v>98</v>
       </c>
       <c r="O23" t="inlineStr"/>
       <c r="P23" t="n">
         <v>0</v>
       </c>
       <c r="Q23" t="n">
-        <v>60</v>
+        <v>98</v>
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>RCM(3)</t>
+          <t>LCB(2)</t>
         </is>
       </c>
       <c r="S23" t="n">
-        <v>60</v>
+        <v>98</v>
       </c>
       <c r="T23" t="inlineStr"/>
       <c r="U23" t="inlineStr"/>
@@ -4781,32 +4797,32 @@
         <v>0</v>
       </c>
       <c r="AF23" t="n">
-        <v>-0</v>
+        <v>0.4</v>
       </c>
       <c r="AG23" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AH23" t="inlineStr">
         <is>
-          <t>Dani Olmo</t>
+          <t>Aymeric Laporte</t>
         </is>
       </c>
       <c r="AI23" t="n">
-        <v>1.1951271</v>
+        <v>1.68469341</v>
       </c>
       <c r="AJ23" t="inlineStr">
         <is>
-          <t>+0.75</t>
+          <t>+1.18</t>
         </is>
       </c>
       <c r="AK23" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="AL23" t="n">
         <v>0</v>
       </c>
       <c r="AM23" t="n">
-        <v>60</v>
+        <v>98</v>
       </c>
       <c r="AN23" t="n">
         <v>0</v>
@@ -4815,19 +4831,19 @@
         <v>1</v>
       </c>
       <c r="AP23" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AQ23" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR23" t="n">
+        <v>2</v>
+      </c>
+      <c r="AS23" t="n">
         <v>3</v>
       </c>
-      <c r="AR23" t="n">
-        <v>2</v>
-      </c>
-      <c r="AS23" t="n">
-        <v>0</v>
-      </c>
       <c r="AT23" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AU23" t="n">
         <v>1</v>
@@ -4858,17 +4874,17 @@
       </c>
       <c r="BD23" t="inlineStr">
         <is>
-          <t>MID</t>
+          <t>DEF</t>
         </is>
       </c>
       <c r="BE23" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="BF23" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="BG23" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
     </row>
     <row r="24">
@@ -4884,17 +4900,17 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Pedri</t>
+          <t>Dani Olmo</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 20</t>
+          <t xml:space="preserve"> 10</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>LCM(3)</t>
+          <t>RCM(3)</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -4904,18 +4920,20 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>4ftlhtels58lyzfluwofzwxuy</t>
-        </is>
-      </c>
-      <c r="I24" t="inlineStr"/>
+          <t>4gq1u1mqg0qzekh1u5djleeax</t>
+        </is>
+      </c>
+      <c r="I24" t="n">
+        <v>2</v>
+      </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
       <c r="K24" t="inlineStr"/>
@@ -4926,22 +4944,22 @@
         </is>
       </c>
       <c r="N24" t="n">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="O24" t="inlineStr"/>
       <c r="P24" t="n">
         <v>0</v>
       </c>
       <c r="Q24" t="n">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="R24" t="inlineStr">
         <is>
-          <t>LCM(3)</t>
+          <t>RCM(3)</t>
         </is>
       </c>
       <c r="S24" t="n">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="T24" t="inlineStr"/>
       <c r="U24" t="inlineStr"/>
@@ -4968,94 +4986,94 @@
         <v>0</v>
       </c>
       <c r="AF24" t="n">
-        <v>0.1</v>
+        <v>-0</v>
       </c>
       <c r="AG24" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AH24" t="inlineStr">
         <is>
-          <t>Pedri</t>
+          <t>Dani Olmo</t>
         </is>
       </c>
       <c r="AI24" t="n">
-        <v>0.74505007</v>
+        <v>1.1951271</v>
       </c>
       <c r="AJ24" t="inlineStr">
         <is>
-          <t>+0.30</t>
+          <t>+0.69</t>
         </is>
       </c>
       <c r="AK24" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="AL24" t="n">
         <v>0</v>
       </c>
       <c r="AM24" t="n">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="AN24" t="n">
         <v>0</v>
       </c>
       <c r="AO24" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AP24" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AQ24" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AR24" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="AS24" t="n">
         <v>0</v>
       </c>
       <c r="AT24" t="n">
+        <v>1</v>
+      </c>
+      <c r="AU24" t="n">
+        <v>1</v>
+      </c>
+      <c r="AV24" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW24" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX24" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY24" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ24" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA24" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB24" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC24" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD24" t="inlineStr">
+        <is>
+          <t>MID</t>
+        </is>
+      </c>
+      <c r="BE24" t="n">
+        <v>4</v>
+      </c>
+      <c r="BF24" t="n">
+        <v>4</v>
+      </c>
+      <c r="BG24" t="n">
         <v>6</v>
-      </c>
-      <c r="AU24" t="n">
-        <v>0</v>
-      </c>
-      <c r="AV24" t="n">
-        <v>1</v>
-      </c>
-      <c r="AW24" t="n">
-        <v>0</v>
-      </c>
-      <c r="AX24" t="n">
-        <v>0</v>
-      </c>
-      <c r="AY24" t="n">
-        <v>0</v>
-      </c>
-      <c r="AZ24" t="n">
-        <v>0</v>
-      </c>
-      <c r="BA24" t="n">
-        <v>0</v>
-      </c>
-      <c r="BB24" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC24" t="n">
-        <v>0</v>
-      </c>
-      <c r="BD24" t="inlineStr">
-        <is>
-          <t>MID</t>
-        </is>
-      </c>
-      <c r="BE24" t="n">
-        <v>12</v>
-      </c>
-      <c r="BF24" t="n">
-        <v>1</v>
-      </c>
-      <c r="BG24" t="n">
-        <v>5</v>
       </c>
     </row>
     <row r="25">
@@ -5071,17 +5089,17 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Mikel Oyarzabal</t>
+          <t>Pedri</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 21</t>
+          <t xml:space="preserve"> 20</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>CF</t>
+          <t>LCM(3)</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -5091,12 +5109,12 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>8</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>b45ryclny991bm7qosieyg1cl</t>
+          <t>4ftlhtels58lyzfluwofzwxuy</t>
         </is>
       </c>
       <c r="I25" t="n">
@@ -5115,22 +5133,22 @@
         </is>
       </c>
       <c r="N25" t="n">
-        <v>45</v>
+        <v>69</v>
       </c>
       <c r="O25" t="inlineStr"/>
       <c r="P25" t="n">
         <v>0</v>
       </c>
       <c r="Q25" t="n">
-        <v>45</v>
+        <v>69</v>
       </c>
       <c r="R25" t="inlineStr">
         <is>
-          <t>CF</t>
+          <t>LCM(3)</t>
         </is>
       </c>
       <c r="S25" t="n">
-        <v>45</v>
+        <v>69</v>
       </c>
       <c r="T25" t="inlineStr"/>
       <c r="U25" t="inlineStr"/>
@@ -5151,68 +5169,68 @@
         </is>
       </c>
       <c r="AD25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="AE25" t="n">
         <v>0</v>
       </c>
       <c r="AF25" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="AG25" t="n">
         <v>2</v>
       </c>
       <c r="AH25" t="inlineStr">
         <is>
-          <t>Mikel Oyarzabal</t>
+          <t>Pedri</t>
         </is>
       </c>
       <c r="AI25" t="n">
-        <v>3.79725599</v>
+        <v>0.7911880400000001</v>
       </c>
       <c r="AJ25" t="inlineStr">
         <is>
-          <t>+3.35</t>
+          <t>+0.28</t>
         </is>
       </c>
       <c r="AK25" t="n">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="AL25" t="n">
         <v>0</v>
       </c>
       <c r="AM25" t="n">
-        <v>90</v>
+        <v>69</v>
       </c>
       <c r="AN25" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AO25" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AP25" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AQ25" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AR25" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AS25" t="n">
         <v>0</v>
       </c>
       <c r="AT25" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="AU25" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AV25" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AW25" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AX25" t="n">
         <v>0</v>
@@ -5234,17 +5252,17 @@
       </c>
       <c r="BD25" t="inlineStr">
         <is>
-          <t>FWD</t>
+          <t>MID</t>
         </is>
       </c>
       <c r="BE25" t="n">
+        <v>12</v>
+      </c>
+      <c r="BF25" t="n">
+        <v>1</v>
+      </c>
+      <c r="BG25" t="n">
         <v>5</v>
-      </c>
-      <c r="BF25" t="n">
-        <v>4</v>
-      </c>
-      <c r="BG25" t="n">
-        <v>12</v>
       </c>
     </row>
     <row r="26">
@@ -5260,17 +5278,17 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Lamine Yamal</t>
+          <t>Mikel Oyarzabal</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 19</t>
+          <t xml:space="preserve"> 21</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>RW</t>
+          <t>CF</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -5280,12 +5298,12 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>9</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>abr79wsl0folgkyvl821ggs2c</t>
+          <t>b45ryclny991bm7qosieyg1cl</t>
         </is>
       </c>
       <c r="I26" t="n">
@@ -5315,7 +5333,7 @@
       </c>
       <c r="R26" t="inlineStr">
         <is>
-          <t>RW</t>
+          <t>CF</t>
         </is>
       </c>
       <c r="S26" t="n">
@@ -5353,19 +5371,19 @@
       </c>
       <c r="AH26" t="inlineStr">
         <is>
-          <t>Lamine Yamal</t>
+          <t>Mikel Oyarzabal</t>
         </is>
       </c>
       <c r="AI26" t="n">
-        <v>2.66864921</v>
+        <v>3.79725599</v>
       </c>
       <c r="AJ26" t="inlineStr">
         <is>
-          <t>+2.22</t>
+          <t>+3.29</t>
         </is>
       </c>
       <c r="AK26" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AL26" t="n">
         <v>0</v>
@@ -5374,34 +5392,34 @@
         <v>90</v>
       </c>
       <c r="AN26" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AO26" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AP26" t="n">
         <v>1</v>
       </c>
       <c r="AQ26" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR26" t="n">
+        <v>4</v>
+      </c>
+      <c r="AS26" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT26" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU26" t="n">
+        <v>1</v>
+      </c>
+      <c r="AV26" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW26" t="n">
         <v>3</v>
-      </c>
-      <c r="AR26" t="n">
-        <v>3</v>
-      </c>
-      <c r="AS26" t="n">
-        <v>1</v>
-      </c>
-      <c r="AT26" t="n">
-        <v>0</v>
-      </c>
-      <c r="AU26" t="n">
-        <v>1</v>
-      </c>
-      <c r="AV26" t="n">
-        <v>0</v>
-      </c>
-      <c r="AW26" t="n">
-        <v>2</v>
       </c>
       <c r="AX26" t="n">
         <v>0</v>
@@ -5430,10 +5448,10 @@
         <v>5</v>
       </c>
       <c r="BF26" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="BG26" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
     </row>
     <row r="27">
@@ -5449,17 +5467,17 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Álex Baena</t>
+          <t>Lamine Yamal</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 15</t>
+          <t xml:space="preserve"> 19</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>LW</t>
+          <t>RW</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -5469,12 +5487,12 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>10</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>5zoz3mjooujpv0wdcphyrztd6</t>
+          <t>abr79wsl0folgkyvl821ggs2c</t>
         </is>
       </c>
       <c r="I27" t="n">
@@ -5493,22 +5511,22 @@
         </is>
       </c>
       <c r="N27" t="n">
-        <v>61</v>
+        <v>45</v>
       </c>
       <c r="O27" t="inlineStr"/>
       <c r="P27" t="n">
         <v>0</v>
       </c>
       <c r="Q27" t="n">
-        <v>61</v>
+        <v>45</v>
       </c>
       <c r="R27" t="inlineStr">
         <is>
-          <t>LW</t>
+          <t>RW</t>
         </is>
       </c>
       <c r="S27" t="n">
-        <v>61</v>
+        <v>45</v>
       </c>
       <c r="T27" t="inlineStr"/>
       <c r="U27" t="inlineStr"/>
@@ -5529,7 +5547,7 @@
         </is>
       </c>
       <c r="AD27" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AE27" t="n">
         <v>0</v>
@@ -5542,55 +5560,55 @@
       </c>
       <c r="AH27" t="inlineStr">
         <is>
-          <t>Álex Baena</t>
+          <t>Lamine Yamal</t>
         </is>
       </c>
       <c r="AI27" t="n">
-        <v>1.09133033</v>
+        <v>2.66864921</v>
       </c>
       <c r="AJ27" t="inlineStr">
         <is>
-          <t>+0.65</t>
+          <t>+2.16</t>
         </is>
       </c>
       <c r="AK27" t="n">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="AL27" t="n">
         <v>0</v>
       </c>
       <c r="AM27" t="n">
-        <v>61</v>
+        <v>90</v>
       </c>
       <c r="AN27" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AO27" t="n">
         <v>0</v>
       </c>
       <c r="AP27" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AQ27" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AR27" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="AS27" t="n">
         <v>1</v>
       </c>
       <c r="AT27" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AU27" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AV27" t="n">
         <v>0</v>
       </c>
       <c r="AW27" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AX27" t="n">
         <v>0</v>
@@ -5610,15 +5628,19 @@
       <c r="BC27" t="n">
         <v>0</v>
       </c>
-      <c r="BD27" t="inlineStr"/>
+      <c r="BD27" t="inlineStr">
+        <is>
+          <t>FWD</t>
+        </is>
+      </c>
       <c r="BE27" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="BF27" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="BG27" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
     </row>
     <row r="28">
@@ -5634,68 +5656,66 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Mikel Merino</t>
+          <t>Álex Baena</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 6</t>
+          <t xml:space="preserve"> 15</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>RCM(3)</t>
+          <t>LW</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>5zoz3mjooujpv0wdcphyrztd6</t>
+        </is>
+      </c>
+      <c r="I28" t="n">
+        <v>2</v>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr"/>
+      <c r="L28" t="inlineStr"/>
+      <c r="M28" t="inlineStr">
+        <is>
           <t>no</t>
         </is>
       </c>
-      <c r="G28" t="inlineStr">
-        <is>
-          <t>0</t>
-        </is>
-      </c>
-      <c r="H28" t="inlineStr">
-        <is>
-          <t>atigcsq78g14w82lwvay26aj9</t>
-        </is>
-      </c>
-      <c r="I28" t="inlineStr"/>
-      <c r="J28" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="K28" t="n">
-        <v>60</v>
-      </c>
-      <c r="L28" t="n">
-        <v>2</v>
-      </c>
-      <c r="M28" t="inlineStr">
-        <is>
-          <t>yes</t>
-        </is>
-      </c>
       <c r="N28" t="n">
-        <v>5</v>
+        <v>61</v>
       </c>
       <c r="O28" t="inlineStr"/>
       <c r="P28" t="n">
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="Q28" t="n">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="R28" t="inlineStr">
         <is>
-          <t>RCM(3)</t>
+          <t>LW</t>
         </is>
       </c>
       <c r="S28" t="n">
-        <v>5</v>
+        <v>61</v>
       </c>
       <c r="T28" t="inlineStr"/>
       <c r="U28" t="inlineStr"/>
@@ -5716,38 +5736,38 @@
         </is>
       </c>
       <c r="AD28" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="AE28" t="n">
         <v>0</v>
       </c>
       <c r="AF28" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AG28" t="n">
         <v>2</v>
       </c>
       <c r="AH28" t="inlineStr">
         <is>
-          <t>Mikel Merino</t>
+          <t>Álex Baena</t>
         </is>
       </c>
       <c r="AI28" t="n">
-        <v>0.20741612</v>
+        <v>1.09133033</v>
       </c>
       <c r="AJ28" t="inlineStr">
         <is>
-          <t>-0.24</t>
+          <t>+0.58</t>
         </is>
       </c>
       <c r="AK28" t="n">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="AL28" t="n">
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="AM28" t="n">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="AN28" t="n">
         <v>0</v>
@@ -5756,19 +5776,19 @@
         <v>0</v>
       </c>
       <c r="AP28" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AQ28" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AR28" t="n">
         <v>1</v>
       </c>
       <c r="AS28" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AT28" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU28" t="n">
         <v>0</v>
@@ -5802,7 +5822,7 @@
         <v>0</v>
       </c>
       <c r="BF28" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="BG28" t="n">
         <v>0</v>
@@ -5821,17 +5841,17 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Ferran Torres</t>
+          <t>Mikel Merino</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 7</t>
+          <t xml:space="preserve"> 6</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>CF</t>
+          <t>RCM(3)</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -5846,7 +5866,7 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>2szgrzcosfeifh664tgt3mfvt</t>
+          <t>atigcsq78g14w82lwvay26aj9</t>
         </is>
       </c>
       <c r="I29" t="inlineStr"/>
@@ -5856,7 +5876,7 @@
         </is>
       </c>
       <c r="K29" t="n">
-        <v>45</v>
+        <v>60</v>
       </c>
       <c r="L29" t="n">
         <v>2</v>
@@ -5867,22 +5887,22 @@
         </is>
       </c>
       <c r="N29" t="n">
-        <v>20</v>
+        <v>38</v>
       </c>
       <c r="O29" t="inlineStr"/>
       <c r="P29" t="n">
-        <v>45</v>
+        <v>60</v>
       </c>
       <c r="Q29" t="n">
-        <v>65</v>
+        <v>98</v>
       </c>
       <c r="R29" t="inlineStr">
         <is>
-          <t>CF</t>
+          <t>RCM(3)</t>
         </is>
       </c>
       <c r="S29" t="n">
-        <v>20</v>
+        <v>38</v>
       </c>
       <c r="T29" t="inlineStr"/>
       <c r="U29" t="inlineStr"/>
@@ -5903,38 +5923,38 @@
         </is>
       </c>
       <c r="AD29" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AE29" t="n">
         <v>0</v>
       </c>
       <c r="AF29" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AG29" t="n">
         <v>2</v>
       </c>
       <c r="AH29" t="inlineStr">
         <is>
-          <t>Ferran Torres</t>
+          <t>Mikel Merino</t>
         </is>
       </c>
       <c r="AI29" t="n">
-        <v>0.36614293</v>
+        <v>0.1183504</v>
       </c>
       <c r="AJ29" t="inlineStr">
         <is>
-          <t>-0.08</t>
+          <t>-0.39</t>
         </is>
       </c>
       <c r="AK29" t="n">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="AL29" t="n">
-        <v>90</v>
+        <v>60</v>
       </c>
       <c r="AM29" t="n">
-        <v>65</v>
+        <v>98</v>
       </c>
       <c r="AN29" t="n">
         <v>0</v>
@@ -5943,13 +5963,13 @@
         <v>0</v>
       </c>
       <c r="AP29" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AQ29" t="n">
         <v>1</v>
       </c>
       <c r="AR29" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AS29" t="n">
         <v>0</v>
@@ -5964,7 +5984,7 @@
         <v>0</v>
       </c>
       <c r="AW29" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AX29" t="n">
         <v>0</v>
@@ -5984,11 +6004,7 @@
       <c r="BC29" t="n">
         <v>0</v>
       </c>
-      <c r="BD29" t="inlineStr">
-        <is>
-          <t>FWD</t>
-        </is>
-      </c>
+      <c r="BD29" t="inlineStr"/>
       <c r="BE29" t="n">
         <v>0</v>
       </c>
@@ -5996,7 +6012,7 @@
         <v>2</v>
       </c>
       <c r="BG29" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="30">
@@ -6012,17 +6028,17 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Yéremy Pino</t>
+          <t>Ferran Torres</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 11</t>
+          <t xml:space="preserve"> 7</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>RW</t>
+          <t>CF</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -6037,7 +6053,7 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>4eezya3lwcwur6c8s6rl0rzvu</t>
+          <t>2szgrzcosfeifh664tgt3mfvt</t>
         </is>
       </c>
       <c r="I30" t="inlineStr"/>
@@ -6058,22 +6074,22 @@
         </is>
       </c>
       <c r="N30" t="n">
-        <v>20</v>
+        <v>53</v>
       </c>
       <c r="O30" t="inlineStr"/>
       <c r="P30" t="n">
         <v>45</v>
       </c>
       <c r="Q30" t="n">
-        <v>65</v>
+        <v>98</v>
       </c>
       <c r="R30" t="inlineStr">
         <is>
-          <t>RW</t>
+          <t>CF</t>
         </is>
       </c>
       <c r="S30" t="n">
-        <v>20</v>
+        <v>53</v>
       </c>
       <c r="T30" t="inlineStr"/>
       <c r="U30" t="inlineStr"/>
@@ -6107,25 +6123,25 @@
       </c>
       <c r="AH30" t="inlineStr">
         <is>
-          <t>Yéremy Pino</t>
+          <t>Ferran Torres</t>
         </is>
       </c>
       <c r="AI30" t="n">
-        <v>-0.1396171</v>
+        <v>0.32459795</v>
       </c>
       <c r="AJ30" t="inlineStr">
         <is>
-          <t>-0.58</t>
+          <t>-0.18</t>
         </is>
       </c>
       <c r="AK30" t="n">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="AL30" t="n">
         <v>90</v>
       </c>
       <c r="AM30" t="n">
-        <v>65</v>
+        <v>98</v>
       </c>
       <c r="AN30" t="n">
         <v>0</v>
@@ -6137,10 +6153,10 @@
         <v>0</v>
       </c>
       <c r="AQ30" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AR30" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AS30" t="n">
         <v>0</v>
@@ -6155,7 +6171,7 @@
         <v>0</v>
       </c>
       <c r="AW30" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AX30" t="n">
         <v>0</v>
@@ -6175,7 +6191,11 @@
       <c r="BC30" t="n">
         <v>0</v>
       </c>
-      <c r="BD30" t="inlineStr"/>
+      <c r="BD30" t="inlineStr">
+        <is>
+          <t>FWD</t>
+        </is>
+      </c>
       <c r="BE30" t="n">
         <v>0</v>
       </c>
@@ -6183,7 +6203,7 @@
         <v>2</v>
       </c>
       <c r="BG30" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="31">
@@ -6199,17 +6219,17 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Nico Williams</t>
+          <t>Fabián Ruiz</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t xml:space="preserve"> 17</t>
+          <t xml:space="preserve"> 8</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>LW</t>
+          <t>LCM(3)</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -6224,7 +6244,7 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>66jotyvbhtz5cjvhbby6luelm</t>
+          <t>f3v58fkymhrprt5gs0ccm29xx</t>
         </is>
       </c>
       <c r="I31" t="inlineStr"/>
@@ -6234,7 +6254,7 @@
         </is>
       </c>
       <c r="K31" t="n">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="L31" t="n">
         <v>2</v>
@@ -6245,22 +6265,22 @@
         </is>
       </c>
       <c r="N31" t="n">
-        <v>4</v>
+        <v>29</v>
       </c>
       <c r="O31" t="inlineStr"/>
       <c r="P31" t="n">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="Q31" t="n">
-        <v>65</v>
+        <v>98</v>
       </c>
       <c r="R31" t="inlineStr">
         <is>
-          <t>LW</t>
+          <t>LCM(3)</t>
         </is>
       </c>
       <c r="S31" t="n">
-        <v>4</v>
+        <v>29</v>
       </c>
       <c r="T31" t="inlineStr"/>
       <c r="U31" t="inlineStr"/>
@@ -6287,93 +6307,471 @@
         <v>0</v>
       </c>
       <c r="AF31" t="n">
-        <v>0</v>
+        <v>-0</v>
       </c>
       <c r="AG31" t="n">
         <v>2</v>
       </c>
       <c r="AH31" t="inlineStr">
         <is>
+          <t>Fabián Ruiz</t>
+        </is>
+      </c>
+      <c r="AI31" t="n">
+        <v>0.36255889</v>
+      </c>
+      <c r="AJ31" t="inlineStr">
+        <is>
+          <t>-0.14</t>
+        </is>
+      </c>
+      <c r="AK31" t="n">
+        <v>13</v>
+      </c>
+      <c r="AL31" t="n">
+        <v>69</v>
+      </c>
+      <c r="AM31" t="n">
+        <v>98</v>
+      </c>
+      <c r="AN31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP31" t="n">
+        <v>1</v>
+      </c>
+      <c r="AQ31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR31" t="n">
+        <v>2</v>
+      </c>
+      <c r="AS31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY31" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ31" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA31" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB31" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC31" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD31" t="inlineStr">
+        <is>
+          <t>MID</t>
+        </is>
+      </c>
+      <c r="BE31" t="n">
+        <v>2</v>
+      </c>
+      <c r="BF31" t="n">
+        <v>1</v>
+      </c>
+      <c r="BG31" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>8muyl6d5ahy04fbwarplcg3kk</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>eh7yt2x2wck51oixw8012ux5j</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Yéremy Pino</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 11</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>RW</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>4eezya3lwcwur6c8s6rl0rzvu</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr"/>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K32" t="n">
+        <v>45</v>
+      </c>
+      <c r="L32" t="n">
+        <v>2</v>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="N32" t="n">
+        <v>53</v>
+      </c>
+      <c r="O32" t="inlineStr"/>
+      <c r="P32" t="n">
+        <v>45</v>
+      </c>
+      <c r="Q32" t="n">
+        <v>98</v>
+      </c>
+      <c r="R32" t="inlineStr">
+        <is>
+          <t>RW</t>
+        </is>
+      </c>
+      <c r="S32" t="n">
+        <v>53</v>
+      </c>
+      <c r="T32" t="inlineStr"/>
+      <c r="U32" t="inlineStr"/>
+      <c r="V32" t="inlineStr"/>
+      <c r="W32" t="inlineStr"/>
+      <c r="X32" t="inlineStr"/>
+      <c r="Y32" t="inlineStr"/>
+      <c r="Z32" t="inlineStr"/>
+      <c r="AA32" t="inlineStr"/>
+      <c r="AB32" t="inlineStr">
+        <is>
+          <t>eh7yt2x2wck51oixw8012ux5j</t>
+        </is>
+      </c>
+      <c r="AC32" t="inlineStr">
+        <is>
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="AD32" t="n">
+        <v>1</v>
+      </c>
+      <c r="AE32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG32" t="n">
+        <v>2</v>
+      </c>
+      <c r="AH32" t="inlineStr">
+        <is>
+          <t>Yéremy Pino</t>
+        </is>
+      </c>
+      <c r="AI32" t="n">
+        <v>-0.04585396000000003</v>
+      </c>
+      <c r="AJ32" t="inlineStr">
+        <is>
+          <t>-0.55</t>
+        </is>
+      </c>
+      <c r="AK32" t="n">
+        <v>21</v>
+      </c>
+      <c r="AL32" t="n">
+        <v>90</v>
+      </c>
+      <c r="AM32" t="n">
+        <v>98</v>
+      </c>
+      <c r="AN32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ32" t="n">
+        <v>2</v>
+      </c>
+      <c r="AR32" t="n">
+        <v>1</v>
+      </c>
+      <c r="AS32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY32" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ32" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA32" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB32" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC32" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD32" t="inlineStr"/>
+      <c r="BE32" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF32" t="n">
+        <v>2</v>
+      </c>
+      <c r="BG32" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>8muyl6d5ahy04fbwarplcg3kk</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>eh7yt2x2wck51oixw8012ux5j</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
           <t>Nico Williams</t>
         </is>
       </c>
-      <c r="AI31" t="n">
-        <v>-0.009421580000000002</v>
-      </c>
-      <c r="AJ31" t="inlineStr">
-        <is>
-          <t>-0.45</t>
-        </is>
-      </c>
-      <c r="AK31" t="n">
-        <v>19</v>
-      </c>
-      <c r="AL31" t="n">
+      <c r="D33" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> 17</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>LW</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>66jotyvbhtz5cjvhbby6luelm</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr"/>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="K33" t="n">
         <v>61</v>
       </c>
-      <c r="AM31" t="n">
-        <v>65</v>
-      </c>
-      <c r="AN31" t="n">
-        <v>0</v>
-      </c>
-      <c r="AO31" t="n">
-        <v>0</v>
-      </c>
-      <c r="AP31" t="n">
-        <v>0</v>
-      </c>
-      <c r="AQ31" t="n">
-        <v>0</v>
-      </c>
-      <c r="AR31" t="n">
-        <v>0</v>
-      </c>
-      <c r="AS31" t="n">
-        <v>0</v>
-      </c>
-      <c r="AT31" t="n">
-        <v>0</v>
-      </c>
-      <c r="AU31" t="n">
-        <v>0</v>
-      </c>
-      <c r="AV31" t="n">
-        <v>0</v>
-      </c>
-      <c r="AW31" t="n">
-        <v>0</v>
-      </c>
-      <c r="AX31" t="n">
-        <v>0</v>
-      </c>
-      <c r="AY31" t="n">
-        <v>0</v>
-      </c>
-      <c r="AZ31" t="n">
-        <v>0</v>
-      </c>
-      <c r="BA31" t="n">
-        <v>0</v>
-      </c>
-      <c r="BB31" t="n">
-        <v>0</v>
-      </c>
-      <c r="BC31" t="n">
-        <v>0</v>
-      </c>
-      <c r="BD31" t="inlineStr">
+      <c r="L33" t="n">
+        <v>2</v>
+      </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="N33" t="n">
+        <v>37</v>
+      </c>
+      <c r="O33" t="inlineStr"/>
+      <c r="P33" t="n">
+        <v>61</v>
+      </c>
+      <c r="Q33" t="n">
+        <v>98</v>
+      </c>
+      <c r="R33" t="inlineStr">
+        <is>
+          <t>LW</t>
+        </is>
+      </c>
+      <c r="S33" t="n">
+        <v>37</v>
+      </c>
+      <c r="T33" t="inlineStr"/>
+      <c r="U33" t="inlineStr"/>
+      <c r="V33" t="inlineStr"/>
+      <c r="W33" t="inlineStr"/>
+      <c r="X33" t="inlineStr"/>
+      <c r="Y33" t="inlineStr"/>
+      <c r="Z33" t="inlineStr"/>
+      <c r="AA33" t="inlineStr"/>
+      <c r="AB33" t="inlineStr">
+        <is>
+          <t>eh7yt2x2wck51oixw8012ux5j</t>
+        </is>
+      </c>
+      <c r="AC33" t="inlineStr">
+        <is>
+          <t>Spain</t>
+        </is>
+      </c>
+      <c r="AD33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AF33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AG33" t="n">
+        <v>2</v>
+      </c>
+      <c r="AH33" t="inlineStr">
+        <is>
+          <t>Nico Williams</t>
+        </is>
+      </c>
+      <c r="AI33" t="n">
+        <v>-0.16098294</v>
+      </c>
+      <c r="AJ33" t="inlineStr">
+        <is>
+          <t>-0.67</t>
+        </is>
+      </c>
+      <c r="AK33" t="n">
+        <v>25</v>
+      </c>
+      <c r="AL33" t="n">
+        <v>61</v>
+      </c>
+      <c r="AM33" t="n">
+        <v>98</v>
+      </c>
+      <c r="AN33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AO33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AP33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AQ33" t="n">
+        <v>2</v>
+      </c>
+      <c r="AR33" t="n">
+        <v>1</v>
+      </c>
+      <c r="AS33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AT33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY33" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ33" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA33" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB33" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC33" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD33" t="inlineStr">
         <is>
           <t>FWD</t>
         </is>
       </c>
-      <c r="BE31" t="n">
-        <v>0</v>
-      </c>
-      <c r="BF31" t="n">
-        <v>0</v>
-      </c>
-      <c r="BG31" t="n">
+      <c r="BE33" t="n">
+        <v>1</v>
+      </c>
+      <c r="BF33" t="n">
+        <v>2</v>
+      </c>
+      <c r="BG33" t="n">
         <v>1</v>
       </c>
     </row>

</xml_diff>